<commit_message>
Refine sublineage definitions and sublineage build layer
</commit_message>
<xml_diff>
--- a/tabular/reference/herv_reference_feature_locations_sublineage.xlsx
+++ b/tabular/reference/herv_reference_feature_locations_sublineage.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A72E5C-43B8-5B46-B52A-7CA7F92271F5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602AE1FE-F833-9349-999E-4AD09D9135DD}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="940" yWindow="500" windowWidth="27860" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="32">
   <si>
     <t>referenceName</t>
   </si>
@@ -54,9 +54,6 @@
     <t>Zetaretrovirus</t>
   </si>
   <si>
-    <t>Gammaretrovirus</t>
-  </si>
-  <si>
     <t>Lambdaretrovirus</t>
   </si>
   <si>
@@ -69,9 +66,6 @@
     <t>ERV3-16A3</t>
   </si>
   <si>
-    <t>HERV-1</t>
-  </si>
-  <si>
     <t>HERV-16</t>
   </si>
   <si>
@@ -94,9 +88,6 @@
   </si>
   <si>
     <t>whole_genome</t>
-  </si>
-  <si>
-    <t>REF_HERV1</t>
   </si>
   <si>
     <t>REF_HERV16</t>
@@ -2379,7 +2370,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C3E50F8-B3B1-CA4C-9209-3ED223B19FBF}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31.33203125" customWidth="1"/>
@@ -2400,7 +2391,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -2411,94 +2402,94 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2">
-        <v>9611</v>
+        <v>9084</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
         <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3">
-        <v>9084</v>
+        <v>933</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4">
-        <v>933</v>
+        <v>7048</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
         <v>6</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5">
-        <v>7048</v>
+        <v>6918</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -2506,16 +2497,16 @@
         <v>28</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6">
-        <v>6918</v>
+        <v>4981</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
@@ -2526,19 +2517,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7">
-        <v>4981</v>
+        <v>7133</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -2549,19 +2540,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8">
-        <v>7133</v>
+        <v>2880</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -2572,71 +2563,48 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9">
-        <v>2880</v>
+        <v>4996</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F9" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10">
-        <v>4996</v>
+        <v>6070</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F10" t="s">
         <v>7</v>
       </c>
       <c r="G10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-      <c r="D11">
-        <v>6070</v>
-      </c>
-      <c r="E11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>